<commit_message>
PDF versions of SI tables
</commit_message>
<xml_diff>
--- a/data/final_tables /Table_S3.xlsx
+++ b/data/final_tables /Table_S3.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anthonyfuentes/Desktop/Submission/data/geochronology/final_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anthonyfuentes/GitHub/Sed_Hematite_UPb/data/final_tables /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF48C6EA-CE87-4C43-B0A6-1BE9AAC24E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D98FCA3B-F5BC-9945-8F4B-2F4E8C16D4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{983A3024-F279-4749-8013-AF771CBD574B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{983A3024-F279-4749-8013-AF771CBD574B}"/>
   </bookViews>
   <sheets>
     <sheet name="U_Pb_data" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">U_Pb_data!$A$1:$Q$513</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -22575,6 +22578,6 @@
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup scale="39" fitToHeight="10" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup scale="41" fitToHeight="10" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>